<commit_message>
Melhorando visual e cálculos da planilha
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Relatório de Vendas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +27,35 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+        <bgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +63,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,49 +455,110 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Produto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Preço</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Quantidade</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>100</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Teclado</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="n">
         <v>150</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Monitor</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>900</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Total Geral</t>
+        </is>
+      </c>
+      <c r="D6" s="5">
+        <f>SUM(D2:D5)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adicionando gráfico automático de vendas
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Relatório de Vendas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relatório de Vendas'!$A$1:$D$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -35,7 +37,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +48,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
         <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -73,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -84,10 +92,13 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -164,6 +175,145 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Vendas por Produto</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Relatório de Vendas'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Relatório de Vendas'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Relatório de Vendas'!$D$2:$D$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Produtos</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Valor Total</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -455,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -530,7 +680,7 @@
       <c r="C4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="4" t="n">
         <v>2700</v>
       </c>
     </row>
@@ -546,22 +696,31 @@
       <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="4" t="n">
         <v>3500</v>
       </c>
     </row>
     <row r="6">
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Total Geral</t>
         </is>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="6">
         <f>SUM(D2:D5)</f>
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Relatório gerado em: 25/05/2026 11:32</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:D5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adicionando gráfico de pizza ao relatório
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -289,6 +289,58 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Participação nas Vendas</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Relatório de Vendas'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Relatório de Vendas'!$D$2:$D$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -308,6 +360,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -714,7 +788,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 25/05/2026 11:32</t>
+          <t>Relatório gerado em: 25/05/2026 11:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Melhorando visual da linha de total geral
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Relatório de Vendas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relatório de Vendas'!$A$1:$D$5</definedName>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +36,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="16"/>
     </font>
   </fonts>
   <fills count="5">
@@ -81,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -101,6 +106,7 @@
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -202,11 +208,6 @@
         <ser>
           <idx val="0"/>
           <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Relatório de Vendas'!D1</f>
-            </strRef>
-          </tx>
           <spPr>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -713,65 +714,65 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Notebook</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>100</v>
+        <v>3500</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>200</v>
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>3500</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>150</v>
+        <v>900</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>150</v>
+        <v>3</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>2700</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>900</v>
+        <v>100</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>2700</v>
+        <v>2</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Notebook</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>3500</v>
+        <v>150</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="4" t="n">
-        <v>3500</v>
+      <c r="D5" s="3" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="6">
@@ -788,7 +789,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 25/05/2026 11:57</t>
+          <t>Relatório gerado em: 27/05/2026 14:37</t>
         </is>
       </c>
     </row>
@@ -797,4 +798,35 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>RESUMO EXECUTIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Quantidade de Produtos</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adicionando exportação automática de relatório em texto
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,13 +36,10 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
       <sz val="16"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -57,8 +54,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00F4CCCC"/>
+        <bgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -86,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -100,13 +103,16 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -739,7 +745,7 @@
       <c r="C3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>2700</v>
       </c>
     </row>
@@ -776,12 +782,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Total Geral</t>
         </is>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="7">
         <f>SUM(D2:D5)</f>
         <v/>
       </c>
@@ -789,7 +795,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 27/05/2026 14:37</t>
+          <t>Relatório gerado em: 29/05/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -810,7 +816,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>RESUMO EXECUTIVO</t>
         </is>

</xml_diff>

<commit_message>
Expandindo conjunto de dados do relatório
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relatório de Vendas'!$A$1:$D$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relatório de Vendas'!$A$1:$D$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,9 @@
     <font>
       <b val="1"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -89,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -113,6 +116,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -221,12 +226,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Relatório de Vendas'!$A$2:$A$5</f>
+              <f>'Relatório de Vendas'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Relatório de Vendas'!$D$2:$D$5</f>
+              <f>'Relatório de Vendas'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -327,12 +332,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Relatório de Vendas'!$A$2:$A$5</f>
+              <f>'Relatório de Vendas'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Relatório de Vendas'!$D$2:$D$5</f>
+              <f>'Relatório de Vendas'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -686,10 +691,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -720,87 +725,215 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Notebook</t>
+          <t>Notebook Lenovo</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>3500</v>
+        <v>3800</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>3500</v>
+        <v>15200</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Notebook Dell</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>900</v>
+        <v>4200</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="5" t="n">
-        <v>2700</v>
+      <c r="D3" s="4" t="n">
+        <v>12600</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>SSD 1TB</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>200</v>
+        <v>18</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>8100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Memória RAM 16GB</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>150</v>
+        <v>320</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>150</v>
+        <v>25</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>8000</v>
       </c>
     </row>
     <row r="6">
-      <c r="C6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Monitor 24</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Monitor 27</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Cadeira Gamer</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>950</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>5700</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Placa de Vídeo RTX 4060</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Webcam Full HD</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Headset Gamer</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>3360</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Mouse Gamer</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Total Geral</t>
         </is>
       </c>
-      <c r="D6" s="7">
-        <f>SUM(D2:D5)</f>
+      <c r="D14" s="7">
+        <f>SUM(D2:D13)</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Relatório gerado em: 31/05/2026 13:23</t>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Relatório gerado em: 02/06/2026 13:40</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D5"/>
+  <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -812,7 +945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -823,13 +956,45 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Quantidade de Produtos</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Faturamento Total</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>81060</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Produto Destaque</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Notebook Lenovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Quantidade Vendida</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Melhorando visual do resumo executivo
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -36,6 +36,7 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="16"/>
     </font>
     <font>
@@ -116,7 +117,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -995,7 +996,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 06/06/2026 11:04</t>
+          <t>Relatório gerado em: 07/06/2026 18:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implementando ranking de produtos por faturamento
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Relatório de Vendas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ranking" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relatório de Vendas'!$A$1:$E$13</definedName>
@@ -93,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -107,18 +108,19 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -783,12 +785,12 @@
       <c r="C4" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="5" t="n">
         <v>8100</v>
       </c>
     </row>
@@ -804,12 +806,12 @@
       <c r="C5" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="5" t="n">
         <v>8000</v>
       </c>
     </row>
@@ -909,12 +911,12 @@
       <c r="C10" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="5" t="n">
         <v>3600</v>
       </c>
     </row>
@@ -930,12 +932,12 @@
       <c r="C11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="5" t="n">
         <v>3500</v>
       </c>
     </row>
@@ -951,12 +953,12 @@
       <c r="C12" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="5" t="n">
         <v>3360</v>
       </c>
     </row>
@@ -972,31 +974,31 @@
       <c r="C13" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="5" t="n">
         <v>1800</v>
       </c>
     </row>
     <row r="14">
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Total Geral</t>
         </is>
       </c>
-      <c r="D14" s="7">
-        <f>SUM(E2:D13)</f>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="8">
+        <f>SUM(E2:E13)</f>
         <v/>
       </c>
-      <c r="E14" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 07/06/2026 18:50</t>
+          <t>Relatório gerado em: 10/06/2026 11:01</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1041,7 @@
           <t>Faturamento Total</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="11" t="n">
         <v>81060</v>
       </c>
     </row>
@@ -1091,6 +1093,167 @@
         <is>
           <t>3. SSD 1TB</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Notebook Lenovo</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n">
+        <v>15200</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>🥇</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>12600</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>🥈</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>8100</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>🥉</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Memória RAM 16GB</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Monitor 24</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Monitor 27</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cadeira Gamer</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>5700</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Placa de Vídeo RTX 4060</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Webcam Full HD</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Headset Gamer</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>3360</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mouse Gamer</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>1800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adicionando data de geração ao resumo
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -998,7 +998,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 10/06/2026 11:01</t>
+          <t>Relatório gerado em: 11/06/2026 20:13</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1092,6 +1092,18 @@
       <c r="A11" t="inlineStr">
         <is>
           <t>3. SSD 1TB</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Gerado em:</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11/06/2026 20:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adicionando indicador de estoque crítico ao resumo
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -998,7 +998,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 11/06/2026 20:13</t>
+          <t>Relatório gerado em: 12/06/2026 12:15</t>
         </is>
       </c>
     </row>
@@ -1067,6 +1067,16 @@
         <v>128</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Produtos Críticos</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+    </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
@@ -1103,7 +1113,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11/06/2026 20:13</t>
+          <t>12/06/2026 12:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Melhorando layout da aba ranking
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -998,7 +998,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 12/06/2026 12:15</t>
+          <t>Relatório gerado em: 13/06/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>12/06/2026 12:15</t>
+          <t>13/06/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -1130,6 +1130,11 @@
   </sheetPr>
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Centralizando cabeçalhos da aba ranking
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -121,6 +121,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -998,7 +1001,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 13/06/2026 15:22</t>
+          <t>Relatório gerado em: 14/06/2026 23:46</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1116,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>13/06/2026 15:22</t>
+          <t>14/06/2026 23:46</t>
         </is>
       </c>
     </row>
@@ -1137,12 +1140,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Produto</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Faturamento</t>
         </is>

</xml_diff>

<commit_message>
Destacando produto líder no ranking
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -124,6 +124,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1001,7 +1003,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 14/06/2026 23:46</t>
+          <t>Relatório gerado em: 16/06/2026 11:01</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1118,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14/06/2026 23:46</t>
+          <t>16/06/2026 11:01</t>
         </is>
       </c>
     </row>
@@ -1152,15 +1154,15 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>Notebook Lenovo</t>
         </is>
       </c>
-      <c r="B2" s="11" t="n">
+      <c r="B2" s="14" t="n">
         <v>15200</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>🥇</t>
         </is>

</xml_diff>

<commit_message>
Adicionando aba de indicadores de vendas
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Relatório de Vendas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Ranking" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Indicadores" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Indicadores1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relatório de Vendas'!$A$1:$E$13</definedName>
@@ -700,7 +702,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1003,7 +1005,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 16/06/2026 11:01</t>
+          <t>Relatório gerado em: 17/06/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1120,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16/06/2026 11:01</t>
+          <t>17/06/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1136,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1291,4 +1293,84 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>INDICADORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Ticket Médio</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>633.28125</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Produto Mais Caro</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Produto Mais Barato</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mouse Gamer</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Maior Estoque</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Memória RAM 16GB</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adicionando classificacao de desempenho dos produtos
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -128,6 +128,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1005,7 +1007,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 17/06/2026 10:52</t>
+          <t>Relatório gerado em: 19/06/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1122,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17/06/2026 10:52</t>
+          <t>19/06/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -1154,6 +1156,11 @@
           <t>Faturamento</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Classificação</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -1179,7 +1186,7 @@
       <c r="B3" s="11" t="n">
         <v>12600</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>🥈</t>
         </is>
@@ -1194,7 +1201,7 @@
       <c r="B4" s="11" t="n">
         <v>8100</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>🥉</t>
         </is>
@@ -1209,6 +1216,11 @@
       <c r="B5" s="11" t="n">
         <v>8000</v>
       </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Excelente</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1219,6 +1231,11 @@
       <c r="B6" s="11" t="n">
         <v>7200</v>
       </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Bom</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1229,6 +1246,11 @@
       <c r="B7" s="11" t="n">
         <v>7000</v>
       </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Bom</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1239,6 +1261,11 @@
       <c r="B8" s="11" t="n">
         <v>5700</v>
       </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Bom</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1249,6 +1276,11 @@
       <c r="B9" s="11" t="n">
         <v>5000</v>
       </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Bom</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1259,6 +1291,11 @@
       <c r="B10" s="11" t="n">
         <v>3600</v>
       </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1269,6 +1306,11 @@
       <c r="B11" s="11" t="n">
         <v>3500</v>
       </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1279,6 +1321,11 @@
       <c r="B12" s="11" t="n">
         <v>3360</v>
       </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1288,6 +1335,11 @@
       </c>
       <c r="B13" s="11" t="n">
         <v>1800</v>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adicionando indicador de menor faturamento
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -1007,7 +1007,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 19/06/2026 11:22</t>
+          <t>Relatório gerado em: 23/06/2026 10:01</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>19/06/2026 11:22</t>
+          <t>23/06/2026 10:01</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1422,6 +1422,30 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Produto Mais Rentável</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Notebook Lenovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Menor Faturamento</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mouse Gamer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adicionando aba de controle de estoque
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Ranking" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Indicadores" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Indicadores1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Estoque" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relatório de Vendas'!$A$1:$E$13</definedName>
@@ -96,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -130,6 +131,7 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -704,7 +706,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1007,7 +1009,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 23/06/2026 10:01</t>
+          <t>Relatório gerado em: 24/06/2026 11:09</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1124,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>23/06/2026 10:01</t>
+          <t>24/06/2026 11:09</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1140,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1449,4 +1451,50 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Quantidade</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mouse Gamer</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>